<commit_message>
chore: prepare pinball tech demo branch
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/__tables__.xlsx
+++ b/Configs/GameConfig/Datas/__tables__.xlsx
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="3"/>
   <cols>
     <col width="20.3809523809524" customWidth="1" style="2" min="2" max="2"/>
@@ -1188,66 +1188,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="B5" s="0" t="inlineStr">
-        <is>
-          <t>badminton.TbShuttlecockShotTest</t>
-        </is>
-      </c>
-      <c r="C5" s="0" t="inlineStr">
-        <is>
-          <t>ShuttlecockShotTest</t>
-        </is>
-      </c>
-      <c r="D5" s="0" t="b">
-        <v>1</v>
-      </c>
-      <c r="E5" s="0" t="inlineStr">
-        <is>
-          <t>shuttlecock_shot_test.xlsx</t>
-        </is>
-      </c>
-      <c r="H5" s="0" t="inlineStr">
-        <is>
-          <t>c,s</t>
-        </is>
-      </c>
-      <c r="I5" s="0" t="inlineStr">
-        <is>
-          <t>羽毛球球路最小验证表</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>badminton.TbShuttlecockShot</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>ShuttlecockShot</t>
-        </is>
-      </c>
-      <c r="D6" t="b">
-        <v>1</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>shuttlecock_shot.xlsx</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>c,s</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>??????????</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>